<commit_message>
v10.495 - React Foundations + Branding API + G381 (first React UI live)
</commit_message>
<xml_diff>
--- a/data/staff_register.xlsx
+++ b/data/staff_register.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1438"/>
+  <dimension ref="A1:K1439"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1072,7 +1072,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>300001</t>
+          <t>301500</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>300002</t>
+          <t>301501</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1182,7 +1182,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>300003</t>
+          <t>301502</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1237,7 +1237,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>300004</t>
+          <t>301503</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1292,7 +1292,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>300005</t>
+          <t>301504</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1347,7 +1347,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>300006</t>
+          <t>301505</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1402,7 +1402,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>300007</t>
+          <t>301506</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>300008</t>
+          <t>301507</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>300009</t>
+          <t>301508</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1567,7 +1567,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>300010</t>
+          <t>301509</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -79552,6 +79552,58 @@
       </c>
       <c r="K1438" s="3" t="n">
         <v>42213</v>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="inlineStr">
+        <is>
+          <t>ADMIN001</t>
+        </is>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>System Admin</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>System Administrator</t>
+        </is>
+      </c>
+      <c r="D1439" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="E1439" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="F1439" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="G1439" t="inlineStr">
+        <is>
+          <t>ict</t>
+        </is>
+      </c>
+      <c r="H1439" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="I1439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J1439" t="inlineStr">
+        <is>
+          <t>William Mwanake</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>